<commit_message>
feat: add missing student reg ID check and update form AJAX
Add gap detection for numeric new_student_registration_id in get_student_reg_ids.php, return first missing ID in API responses.
Update payment.php to reuse detected missing registration IDs instead of generating max+1 when gaps exist, adjust label text and styling accordingly.
Refactor AJAX form logic across re_register.php, batchSwap.php, and programProgression.php: add university dropdowns, replace old university-agnostic fetch endpoints with university-aware ones.
Clean up commented-out legacy code across multiple files and fix fetch_students.php to include student_code in its SELECT query.
</commit_message>
<xml_diff>
--- a/Sql/HD prob.xlsx
+++ b/Sql/HD prob.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ims-october-bkps\Sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3818C40D-01AA-4A52-A30B-953EB47178CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4A1E00-CFE8-42BF-96A3-30D644C18E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="692" firstSheet="3" activeTab="6" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
+    <workbookView xWindow="23880" yWindow="630" windowWidth="20730" windowHeight="11040" tabRatio="692" firstSheet="5" activeTab="6" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Payment Data Syucess ECM TO GDM" sheetId="3" r:id="rId2"/>
-    <sheet name="Payment Duplicate error fix" sheetId="4" r:id="rId3"/>
-    <sheet name="Transfered  Progression Checkin" sheetId="5" r:id="rId4"/>
-    <sheet name="POS  and PAGE UPDATE" sheetId="7" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="Payment Data Syucess ECM TO GDM" sheetId="3" state="hidden" r:id="rId2"/>
+    <sheet name="Payment Duplicate error fix" sheetId="4" state="hidden" r:id="rId3"/>
+    <sheet name="Transfered  Progression Checkin" sheetId="5" state="hidden" r:id="rId4"/>
+    <sheet name="POS  and PAGE UPDATE" sheetId="7" state="hidden" r:id="rId5"/>
     <sheet name="HD RESULT CHANGE" sheetId="2" r:id="rId6"/>
     <sheet name="re register" sheetId="12" r:id="rId7"/>
     <sheet name="Sheet3" sheetId="13" r:id="rId8"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="126">
   <si>
     <t>Re-sit</t>
   </si>
@@ -477,6 +477,15 @@
   </si>
   <si>
     <t>5/9/2026 updted</t>
+  </si>
+  <si>
+    <t>Payment New ID Order Missing wID wanna get coreclt</t>
+  </si>
+  <si>
+    <t>add_payment_plan_folder\get_student_reg_ids.php</t>
+  </si>
+  <si>
+    <t>6/9/2026 updted</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1201,6 +1210,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4094,11 +4106,11 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6C46C7F-8851-4D1E-AAA5-68FB05373326}">
-  <dimension ref="A2:L11"/>
+  <dimension ref="A2:L22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="52.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="56.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4191,9 +4203,64 @@
       <c r="B11" s="105"/>
       <c r="C11" s="106"/>
     </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E13" s="119" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="119"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D18" s="82"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="83"/>
+    </row>
+    <row r="19" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D19" s="84"/>
+      <c r="E19" s="93" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" s="85" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D20" s="84"/>
+      <c r="E20" s="93" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" s="85" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D21" s="84"/>
+      <c r="E21" s="93" t="s">
+        <v>125</v>
+      </c>
+      <c r="F21" s="85" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="4:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="86"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="87"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="F3:L3"/>
+    <mergeCell ref="E13:F13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4201,100 +4268,9 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F945C220-D127-489B-A05F-24B39A2383B1}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1">
-        <v>1060</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1041</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1040</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1038</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>1032</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>1030</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1027</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>1023</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>1012</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>1006</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>1004</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>547</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Induction From DB concpet changed  for the Unpaid
</commit_message>
<xml_diff>
--- a/Sql/HD prob.xlsx
+++ b/Sql/HD prob.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ims-october-bkps\Sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4A1E00-CFE8-42BF-96A3-30D644C18E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8624F0B-8815-4616-B06B-3211184AD3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="630" windowWidth="20730" windowHeight="11040" tabRatio="692" firstSheet="5" activeTab="6" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
+    <workbookView xWindow="23880" yWindow="630" windowWidth="20730" windowHeight="11040" tabRatio="692" firstSheet="5" activeTab="5" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -18,10 +18,11 @@
     <sheet name="Payment Duplicate error fix" sheetId="4" state="hidden" r:id="rId3"/>
     <sheet name="Transfered  Progression Checkin" sheetId="5" state="hidden" r:id="rId4"/>
     <sheet name="POS  and PAGE UPDATE" sheetId="7" state="hidden" r:id="rId5"/>
-    <sheet name="HD RESULT CHANGE" sheetId="2" r:id="rId6"/>
+    <sheet name="Induction re-arrange" sheetId="13" r:id="rId6"/>
     <sheet name="re register" sheetId="12" r:id="rId7"/>
-    <sheet name="Sheet3" sheetId="13" r:id="rId8"/>
-    <sheet name="Sheet2" sheetId="6" state="hidden" r:id="rId9"/>
+    <sheet name="HD RESULT" sheetId="2" r:id="rId8"/>
+    <sheet name="New ID Order Missing " sheetId="14" r:id="rId9"/>
+    <sheet name="Sheet2" sheetId="6" state="hidden" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="141">
   <si>
     <t>Re-sit</t>
   </si>
@@ -486,6 +487,51 @@
   </si>
   <si>
     <t>6/9/2026 updted</t>
+  </si>
+  <si>
+    <t>induction_DB_folder\fetch_induction_students_from_db.php</t>
+  </si>
+  <si>
+    <t>send_induction_email_from_db.php</t>
+  </si>
+  <si>
+    <t>induction_email_report.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email log table </t>
+  </si>
+  <si>
+    <t>induction_DB_folder\fetch_induction_email_log.php</t>
+  </si>
+  <si>
+    <t>induction_fl_report_db.php</t>
+  </si>
+  <si>
+    <t>induction_DB_folder\fetch_all_induction_db_students.php</t>
+  </si>
+  <si>
+    <t>induction_scan_db.php</t>
+  </si>
+  <si>
+    <t>induction_DB_folder\fetch_attended_db_students.php</t>
+  </si>
+  <si>
+    <t>induction_manual_attend_db.php</t>
+  </si>
+  <si>
+    <t>induction_scan_db_action.php</t>
+  </si>
+  <si>
+    <t>✅</t>
+  </si>
+  <si>
+    <t xml:space="preserve">induction_from_db_email_send.php </t>
+  </si>
+  <si>
+    <t>07-09-2026 Updated</t>
+  </si>
+  <si>
+    <t>07-09-2026 data</t>
   </si>
 </sst>
 </file>
@@ -680,7 +726,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -1011,11 +1057,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1178,6 +1239,9 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1211,14 +1275,23 @@
     <xf numFmtId="0" fontId="10" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1612,6 +1685,146 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>464910</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>11685</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>322950</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>164145</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="4" name="Ink 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4A0CC73-F6CF-847A-15A8-E5DD3D99645E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="6808560" y="973710"/>
+            <a:ext cx="4125240" cy="1866960"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="4" name="Ink 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4A0CC73-F6CF-847A-15A8-E5DD3D99645E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6799560" y="964710"/>
+              <a:ext cx="4142880" cy="1884600"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>32830</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3114675</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>47685</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="2" name="Ink 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B468251-1AC1-4522-A309-C6B6FF399B95}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="1333500" y="2366455"/>
+            <a:ext cx="3000375" cy="1357880"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="2" name="Ink 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B468251-1AC1-4522-A309-C6B6FF399B95}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1324501" y="2357455"/>
+              <a:ext cx="3018014" cy="1375519"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
@@ -1759,6 +1972,62 @@
   <inkml:trace contextRef="#ctx0" brushRef="#br0">207 889 24575,'-4'9'0,"1"0"0,0 0 0,0 0 0,-2 18 0,-2 9 0,-55 224-714,-32 281 1,79-398 240,7 0 0,6 1 1,26 242-1,-3-247 473,76 264 0,-67-310 0,5-2 0,4-1 0,82 139 0,-103-198-37,3-2-1,0 2 1,2-4-1,0 0 1,2-1-1,49 40 1,-60-56 27,0 0 1,1-2 0,0 0 0,0 0-1,0-1 1,1-1 0,1 0 0,-1-2-1,0 0 1,1 0 0,0-1 0,0-1-1,0-2 1,0 1 0,0-2-1,20-1 1,-10-3 9,0-2 0,0 0 0,0-1 0,27-14 0,-1-2-162,87-57 0,85-82-1134,22-63 607,14-64-767,-146 138 1059,-7-6 0,-6-3 0,-8-5 0,128-313 0,-141 261 9,-10-2 0,-9-3 0,52-364 0,-85 315 226,-19 68 538,-9 153 314,-3 0 1,-12-82-1,12 127-515,1-1 0,-1 1 1,0-1-1,0 1 0,-5-9 1,7 14-117,0 0 1,0 1 0,0 0-1,0-1 1,-1 0 0,1 1 0,-1 0-1,1-1 1,0 1 0,0-1-1,-1 0 1,0 1 0,1 0-1,-1 0 1,1-1 0,0 1-1,-1 0 1,0-1 0,1 1-1,0 0 1,-1 0 0,0 0 0,1 0-1,0 0 1,-1 0 0,0-1-1,0 1 1,1 0 0,0 0-1,-1 0 1,0 1 0,1-1-1,-1 0 1,0 0 0,1 0-1,0 0 1,-1 0 0,0 0 0,1 0-1,-1 1 1,1-1 0,0 1-1,-2-1 1,-3 5 109,1 1 0,-1-1 0,1 0-1,-1 1 1,1 0 0,-4 8 0,-114 247 2470,120-255-2651,-98 242-378,-25 95-1169,-14 89 402,-188 828-1337,247-839 1823,-24 445-1,89-471 367,30-72-918,26-66 812,-28-201 376,3 0-1,2 0 1,2-2 0,32 61 0,-41-94 472,1-1 0,0 0 0,1 0 0,31 32 1,-39-48-234,-1 1 1,1-1 0,0 1 0,0-1-1,1 0 1,-1 0 0,2-2 0,-2 2 0,2-1-1,-1-1 1,0 1 0,0-1 0,1 0-1,-1-1 1,1 0 0,-1 0 0,1 0 0,-1-1-1,1 0 1,0-1 0,7 0 0,-4-1 130,0-2 1,0 1 0,-1-1-1,1-1 1,17-9 0,-3-2-41,23-19-1,26-29 245,68-75 1,55-83-1175,-82 80 576,103-165 0,-191 266 113,-3-2 1,-1-1-1,-2 0 0,-2-2 1,-2 0-1,-2-1 0,-3-1 1,-1 0-1,-2 0 0,-2-1 1,-3 0-1,-3-53 0,-1 80-54,-1-2 0,-2 1 0,0 1 0,-2 0 0,-8-22 0,5 28 0,9 16 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,0 3 0,-1 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 3 0,-35 203 0,16 9 0,9-86 0,-27 336 0,27-5 0,11-460 0,0 0 0,0 0 0,0-1 0,1 2 0,-1-1 0,0 0 0,2 4 0,-1-7 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,8-20 0,14-63-54,21-162 0,-38 209-32,60-559-544,-24-5 290,-24 139 245,-16 437 77,-2 16 42,1-1-1,1 1 1,0 0-1,0-1 0,1 1 1,-1 0-1,2 0 1,3-11-1,-5 18 10,0 0-1,0-1 0,0 1 0,0 0 1,0 0-1,0 0 0,0 1 0,0-2 1,1 1-1,-1 1 0,0-1 0,1 0 1,-2 1-1,2 0 0,-1-1 0,1 0 1,0 1-1,-1 0 0,1 0 0,-1 0 1,0 0-1,1 0 0,-1 0 1,1 0-1,-1 0 0,0 0 0,1 0 1,-1 0-1,0 1 0,1 0 0,-1-1 1,1 0-1,-1 1 0,2 1 0,1 0-38,1 0 0,-1 0-1,0 1 1,0-1 0,-1 1 0,1 0-1,0 0 1,-1 0 0,6 6-1,-7-5 7,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,0 0 0,0 0 0,1 1 0,-2-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,-2-1 0,1 1 0,0-1 0,0 0 0,-4 7 0,-4 7 0,0 0 0,-1 0 0,-20 23 0,18-22 0,-4 3 0,3-4 0,1-1 0,0 2 0,1 0 0,-8 24 0,18-42 0,0 0 0,1 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,1 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,-1-1 0,2 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1-2 0,3 2 0,4 3 0,1-2 0,-1 1 0,1-1 0,-1-1 0,11 3 0,27 3 0,94 6 0,50-15 0,-143-1 0,-2-2 0,1-2 0,49-13 0,-78 15 0,-1-2 0,0 0 0,0 0 0,28-18 0,-36 19 0,0-2 0,1 1 0,-2-1 0,0 0 0,1-1 0,-2 1 0,1-2 0,-1 2 0,6-13 0,-7 12 0,-1-1 0,-1 0 0,1-1 0,-1 1 0,-1 0 0,0 0 0,-1-1 0,1 0 0,-2 0 0,1 0 0,-1 1 0,-2-15 0,1 22 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-2 0 0,1 0 0,0-1 0,0 1 0,1 0 0,-1 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,-3 0 0,-7 1 0,1-1 0,0 1 0,-1 1 0,-18 3 0,25-3 0,-44 6 0,-79 23 0,110-25 0,0 1 0,0 1 0,2 1 0,-1 1 0,0 0 0,1 0 0,-23 21 0,34-27 0,1 1 0,0 1 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 2 0,0-1 0,0 1 0,1-2 0,0 2 0,0 0 0,1 0 0,-3 11 0,3-14 0,1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,1 0 0,-1-1 0,0 1 0,1-1 0,0 1 0,0-1 0,0 0 0,-1 0 0,7 3 0,-4-3 0,0 0 0,0 1 0,0-2 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0-1 0,1 1 0,-1-1 0,0-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0-1 0,6-2 0,3-2 0,1 0 0,-2-2 0,1 0 0,-2 0 0,18-14 0,30-32-45,-2-1 0,-3-3 0,53-73 0,-65 77-108,-3-3 0,-2-1 0,-3-2-1,-3-1 1,-2-2 0,-2-1 0,20-73 0,-26 55-174,-4-1 0,-4-1 0,-4-1 0,1-87-1,-11 68 339,-5 0 1,-36-200-1,25 229-147,-3 2 0,-33-86 1,37 125 85,0-1 0,-2 2 0,-2 0 0,0 1 1,-3 0-1,-29-32 0,46 57 94,-1 1 0,0 0 0,0 1 1,-1-1-1,1 1 0,-1 0 0,-13-6 1,18 11-14,-1-2 0,1 1 0,0 1 0,-1 0 1,1-1-1,0 1 0,-1 0 0,0 0 0,1 0 1,-1 0-1,0 0 0,1 1 0,-1-1 0,1 0 0,0 1 1,-1 1-1,1-2 0,0 1 0,-1 0 0,1 1 1,0-1-1,-1 1 0,1-1 0,0 0 0,1 1 1,-1 0-1,0 0 0,-2 3 0,-7 7 174,1 2 0,0 0 0,1 0 0,-8 18 0,-30 74 387,44-100-590,-68 180-226,-9 73-675,-4 86 15,-28 303-2304,33 347 3079,73-674-130,13-64-713,11-65 696,4-75 180,-17-101 127,0 0-1,0 1 0,2-2 1,11 22-1,-15-32 116,0 1 0,1-1 0,-1 0 0,1 0-1,0-1 1,1 0 0,-1 0 0,1 0 0,0 1 0,0-2 0,0 0 0,1 0 0,-1 0 0,0 0-1,1-1 1,0 0 0,0 0 0,-1 0 0,1 0 0,0-2 0,0 2 0,1-2 0,-1 1 0,0-1-1,0 0 1,8-3 0,2 1 119,-2-1 0,0-1-1,1-1 1,-1 0 0,0-1-1,0-1 1,-1 0 0,0 0-1,18-15 1,59-51-217,86-92-1,-150 139-67,-1-1 0,-1-1 0,-1-1 0,-2-1 0,-1-2 0,-1 1 0,-2-2 0,-1 0 0,-2-2 0,-1 1 0,-2-1 0,-1 0 0,-2-2 0,-1 1 0,3-67 0,-11 77 0,-1 0 0,0 0 0,-3 0 0,0 0 0,-1 1 0,-2 0 0,0-1 0,-19-36 0,26 59 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-2 0,-1 2 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-2 1 0,-1-1 0,2 2 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 1 0,1-1 0,-1 0 0,2 1 0,-2 0 0,1-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,1 0 0,-2 0 0,2 0 0,-2 0 0,1 0 0,1 0 0,-1 1 0,0 0 0,-4 5 0,1 2 0,0-2 0,1 2 0,0-1 0,0 0 0,0 1 0,1-1 0,1 2 0,-1-2 0,2 1 0,-1 1 0,1-2 0,1 1 0,1 17 0,-2-25 0,1 1 0,-1-2 0,1 2 0,0-1 0,-1 1 0,0-2 0,1 2 0,0-2 0,-1 2 0,1-2 0,0 2 0,-1-2 0,2 1 0,-2 1 0,1-2 0,1 1 0,-2 0 0,2-1 0,-2 1 0,2 0 0,-1-1 0,0 1 0,2 0 0,-1 0 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,1 0 0,1 0 0,7-3 0,-1-1 0,0-1 0,0 1 0,10-8 0,-4 0 0,-12 10 0,1-2 0,0 2 0,-1-1 0,1 2 0,6-4 0,-10 5 0,1 1 0,-1 0 0,0-1 0,0 1 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-2 1 0,2-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0 0 0,0-1 0,1 1 0,-2 0 0,2-1 0,-1 1 0,1 2 0,3 1 0,-2 1 0,1-1 0,-2 1 0,2 0 0,-1 0 0,2 6 0,-5-8 0,2 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,0-1 0,1 1 0,-2 0 0,1-1 0,1 0 0,3 2 0,9-1 0,0 1 0,0-3 0,1 1 0,-1-2 0,1 1 0,-1-3 0,0 0 0,0 0 0,0-1 0,0 0 0,-1-2 0,0 0 0,16-9 0,3-3 0,-2-1 0,0-2 0,-1-1 0,43-41 0,-40 30-73,-2-2-1,-1 1 0,-1-3 0,-3-1 1,43-78-1,-42 58-36,-2-1-1,-3-1 1,29-114-1,-27 53-88,-6-1 0,-5-1 0,-2-156 0,-44-369-680,8 392 602,16 201 277,8 55 0,0 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0-1 1,0 1-1,0 0 0,0 0 0,0 0 1,0 0-1,0 0 0,0-1 0,0 1 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,0 0 0,0-1 0,0 1 1,0 0-1,0 0 0,0 0 0,0 0 0,0 0 1,0 0-1,-1 0 0,1 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,-1 0 0,1 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,-1 0 0,1 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,0 0-1,0 0 0,0 0 0,0 0 1,-3 14 115,-1 172 503,4-129-575,2 207-362,7 104-952,8 100 184,51 745-2766,43-5 2196,-80-962 1323,-9-98 333,-20-135 119,1 0 0,7 23 0,-10-36-108,0 0 0,0 0-1,0 1 1,0-1 0,0 0 0,0 0 0,0 0-1,0 0 1,0 0 0,0 0 0,0 0 0,0 0 0,0 0-1,0 0 1,0 0 0,0 1 0,0-1 0,0 0-1,0 0 1,1 0 0,-1 0 0,0 0 0,0 0 0,0 0-1,0 1 1,0-1 0,0 0 0,1 0 0,-1 0-1,0 0 1,0 0 0,0 0 0,0 0 0,0 0-1,0 0 1,0 0 0,0 0 0,0 0 0,0 0 0,0 0-1,1 0 1,-1 0 0,0 0 0,0 0 0,0 0-1,0 0 1,0 0 0,1 0 0,-1 0 0,0 0 0,0 0-1,0 0 1,0-1 0,0 1 0,0 0 0,0 0-1,0 0 1,0 0 0,0 0 0,0 0 0,0 0-1,0-1 1,0 1 0,0 0 0,1 0 0,3-16 703,0-163-385,-5 151-301,-25-438 1996,12 353-1349,-4 2 0,-39-126 0,38 177-383,-3 2 1,-1 0-1,-4 2 0,-50-81 0,49 95-49,-2 1 1,-2 2-1,-2 1 0,-1 1 1,-76-60-1,49 55-253,42 30 107,-35-28 0,55 39-64,-1 1 1,0-2-1,0 1 1,0 1-1,1-1 1,-1 0-1,0 0 1,0 0-1,1 0 1,-1 0-1,0 0 1,1-1-1,0 2 1,-1-2 0,1 2-1,0-2 1,-1 0-1,1 1 1,0 0-1,0 0 1,0-1-1,0 0 1,1-1-14,0 1 0,-1-1 1,2 1-1,-1-1 1,0 1-1,0-1 0,1 1 1,0 0-1,2-4 0,18-19 35,2 1 1,0 1-1,2 0 0,31-20 0,-24 19-46,-27 19-9,91-70 0,119-69 0,-214 143 0,5-3 0,0 1 0,-1-1 0,15-3 0,-20 7 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 1 0,-1 0 0,0-1 0,1 0 0,0 1 0,0 0 0,-1 0 0,0-1 0,1 0 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 1 0,0-2 0,0 1 0,0 0 0,0 0 0,-1 10 0,0-2 0,0 2 0,-3 10 0,2-11 0,0-1 0,1 1 0,-1 0 0,2 0 0,0 13 0,0-21 0,1 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,1 0 0,0-1 0,-1 2 0,1-2 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,1-2 0,-1 2 0,0-2 0,5 3 0,5 1 0,0-2 0,0 0 0,0 0 0,0-1 0,0-1 0,1 0 0,-2 0 0,2-2 0,-1 1 0,0-1 0,0-1 0,-1 0 0,17-7 0,-16 5 0,0-1 0,0 1 0,0-2 0,-1 0 0,0 0 0,0-1 0,-1 0 0,0-1 0,0 0 0,-1-1 0,-1 1 0,10-14 0,-13 13 0,-1 1 0,1 0 0,-1 0 0,-1 0 0,0-1 0,0 1 0,-1 0 0,-1-1 0,1-1 0,-1-10 0,0 15 0,-2 1 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,-2-1 0,-1-4 0,2 7 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,-1 0 0,-5-1 0,5 1 0,-1 2 0,1-1 0,0 0 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 1 0,0-1 0,0 0 0,1 1 0,-5 4 0,1-2 0,0 1 0,1 0 0,0 0 0,0 1 0,1 0 0,-1 0 0,1 1 0,0 0 0,-6 15 0,10-22 0,1 0 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,2 1 0,4 1 0,0 1 0,0-1 0,0-1 0,0 0 0,0 0 0,11 1 0,22 2 0,-1-1 0,0-3 0,1-1 0,0-2 0,58-10 0,-28-2 0,-1-2 0,79-31 0,-123 39 0,-1-2 0,0 0 0,0-1 0,-1-1 0,33-24 0,-54 33 0,1 1 0,0 0 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1-5 0,-2 8 0,-1-1 0,0 0 0,1 1 0,-1-2 0,0 1 0,0 1 0,0-1 0,1 0 0,-1 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-2 0 0,1 0 0,1 0 0,-2 0 0,-3 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,1 1 0,-2 0 0,1 0 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-6 5 0,-2 1 0,0 1 0,1 0 0,-20 20 0,26-22 0,-1 0 0,0 0 0,1 0 0,-6 16 0,9-18 0,0-2 0,0 1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 0 0,1 0 0,2 9 0,-2-12 0,0 0 0,1 1 0,-1-2 0,0 2 0,0-2 0,1 2 0,-1-2 0,1 1 0,-1 1 0,1-2 0,0 1 0,-1 0 0,1 0 0,0 0 0,0-1 0,-1 1 0,2 0 0,-2-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,2 1 0,1-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,2 0 0,6-2 0,10-4 0,0 0 0,-2-2 0,1 0 0,0-1 0,25-17 0,-13 6 0,-1-2 0,38-35 0,-42 31-36,-1-2-1,-2-1 1,-1-1 0,-1-1-1,-1-1 1,-2-1-1,-1-1 1,-2 0-1,-1-1 1,-2 0-1,12-51 1,-11 24-33,-3-1-1,-2 0 1,-3-1-1,-4 1 1,-2-1-1,-7-64 0,-2 57 70,-3 0 0,-3 1 0,-3 0 0,-37-91 0,23 85 0,-3 2 0,-3 1 0,-73-104 0,94 153 0,-1-1 0,-1 3 0,-39-37 0,57 57 0,-2 0 0,1 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-4-1 0,5 2 0,1 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,-1 0 0,0 0 0,0 1 0,1-1 0,0 0 0,-1 0 0,0 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,0 1 0,0 0 0,0 1 0,0 0 0,0 0 0,0-1 0,1 1 0,0 0 0,-1 0 0,0-1 0,0 4 0,0 12 0,0 0 0,3 30 0,15 104 0,22 97-472,33 125-1419,37 125 495,41 109-2296,40 78 2151,679 1907-4055,-719-2194 5465,-41-117 436,-101-259-164,98 230 1971,-90-220-293,-16-32-1768,0 0-1,1 0 1,-1 0-1,0 0 1,0 0-1,0 0 1,0 0-1,0 0 0,0 0 1,0 0-1,0 0 1,0 0-1,0 0 1,0 0-1,0 0 1,0 0-1,1 0 1,-10-19 884,-164-341 4584,-132-165-3747,17 118-1780,-15 11 73,238 313-11,30 37 251,-163-222-143,170 224 100,2-1 0,1-2 0,3 0-1,-22-67 1,43 109-239,-1-1 1,0 2-1,1-1 1,1-1-1,-1 1 1,0 0-1,1-1 1,0 1 0,0 0-1,2-7 1,-1 7-26,1 0 1,0-1 0,0 1-1,1 1 1,-1-1 0,2 0-1,-1 1 1,0-1 0,1 1 0,4-6-1,24-20 2,1 0 0,53-37 0,53-30 0,60-37-503,74-42-1508,73-48 791,-303 197 768,669-437-2675,-14-21 2853,-469 311-805,-72 42 800,-119 98 376,-1-1 0,36-46-1,-71 79 6,0 0-1,0-1 1,-1 1-1,1 0 1,-1-1 0,1 0-1,0-5 1,-2 8-65,0 0 1,0-1 0,1 1 0,-1-1 0,0 0 0,0 1-1,0 0 1,0-1 0,0 1 0,0-1 0,0 1-1,-1 0 1,1-1 0,0 1 0,0-1 0,0 1-1,0 0 1,0-1 0,0 1 0,-1-1 0,1 0-1,0 1 1,-1 0 0,1 0 0,0-1 0,0 1 0,-1-1-1,0 1 1,-2-1 247,1 0-1,-2 1 1,1-1 0,1 1-1,-1-1 1,-1 1-1,1 0 1,1 0 0,-2 1-1,1-1 1,-5 2-1,-148 38 2980,1-1-3197,116-31-380,-68 26 0,90-27-426,1-2-6087</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1">8275 3494 24575</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2">8523 3884 24575,'3'0'0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink6.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-09-07T11:18:08.879"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">111 1740 24575,'-1'0'0,"1"1"0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 1 0,0-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-3 6 0,-9 34 0,2 0 0,-8 61 0,-11 116-265,10 2 1,9 0-1,10 0 0,48 377 0,-35-512 265,4 0 0,3-1 0,5-2 0,51 122 0,-63-178 0,0-1 0,2 0 0,0-1 0,2 0 0,1-1 0,1-1 0,0-1 0,31 25 0,-32-32 0,2-1 0,-1-1 0,1 0 0,1-1 0,0-2 0,1 0 0,0-1 0,0-1 0,0-1 0,40 5 0,-17-7-9,0-1 0,0-3 0,0-2 0,0-2 0,-1-1 0,1-3 0,45-14 0,-12-2-160,-1-3 0,-1-3 0,80-46 0,-61 22 131,-3-4 1,-2-4 0,-3-4-1,88-86 1,-82 60 46,-5-4 0,-3-4 1,79-122-1,-114 145 201,-4-2 1,50-115-1,-77 146-105,-1 1 0,-3-2 1,-2 0-1,-2-1 0,7-83 0,-16 119-105,-1 0 0,-1 0 0,0 1 0,-1-1 0,0 0 0,-1 1 0,-1-1 0,0 1 0,-10-26 0,13 38-1,-1 0 0,1-1-1,0 1 1,-1 0 0,0 0 0,1 0-1,-1 0 1,0 0 0,0 0 0,1 0-1,-1 0 1,0 0 0,0 0 0,0 0-1,0 0 1,0 1 0,0-1 0,0 0-1,-1 1 1,1-1 0,0 1 0,0-1-1,0 1 1,-1 0 0,1-1 0,0 1-1,0 0 1,-1 0 0,1 0 0,0 0-1,-2 0 1,0 2 15,0-1 1,0 1-1,0 0 0,1 0 1,-1 0-1,1 0 0,-1 1 0,1-1 1,0 1-1,0-1 0,0 1 1,0 0-1,-1 3 0,-17 32 146,3 0 0,1 1 0,2 0 0,-14 60 0,-10 56-306,-35 309-1,64-355 74,5 1-1,5 0 1,27 190 0,-18-244 73,2 0 0,3 0 0,40 96 0,-43-125 0,1-1 0,1 0 0,1-1 0,2 0 0,0-2 0,2 0 0,0-1 0,1 0 0,26 19 0,-37-34-3,1 0 1,0 0-1,0-1 1,0 0 0,1-1-1,-1 0 1,1-1-1,1 0 1,15 3-1,-22-6 8,-1-1-1,1 0 1,-1 1-1,1-1 1,-1-1-1,1 1 1,-1-1 0,1 1-1,-1-1 1,1-1-1,-1 1 1,0-1-1,0 1 1,0-1-1,0 0 1,0-1-1,0 1 1,0-1-1,-1 1 1,1-1-1,-1 0 1,0-1-1,0 1 1,0-1-1,0 1 1,3-7 0,5-9 53,-2-1 1,0 0 0,-2 0 0,0 0 0,-1-1 0,-1 0 0,-1-1 0,1-21 0,2-177-101,-10 150 42,0 32 0,4-56 0,-1 94 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,2 0 0,10 13 0,11 39 0,123 479 0,-102-356 0,-5-22 0,74 268 0,-93-364 0,-15-50 0,-4-12 0,-14-93 0,-139-879-515,84-16-1,68 971 516,-1 6 0,1 1 0,0 0 0,1 0 0,1-1 0,1 1 0,8-29 0,-10 42 7,-1 1 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,3 0 0,-1 0 21,0 1-1,0 0 0,0 1 0,0-1 1,0 0-1,-1 1 0,1 0 0,0 0 1,0 0-1,-1 1 0,1-1 0,4 3 1,1 1 29,0 1 0,0-1 1,-1 2-1,1-1 0,-1 1 0,-1 1 1,1-1-1,11 17 0,-13-14-57,-1 0 0,0 0 0,0 1 0,-1 0 0,0 0 0,-1 0 0,0 0 0,-1 1 0,0-1 0,-1 1 0,0 17 0,-2-12 0,-1 0 0,0 0 0,-2 0 0,0-1 0,0 0 0,-2 0 0,-8 18 0,-8 8 0,-1-2 0,-3 0 0,-1-2 0,-56 62 0,38-56 0,35-36 0,0 2 0,0-1 0,1 1 0,0 0 0,1 1 0,0 0 0,-10 19 0,18-29 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1-1 0,1 1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,-1 0 0,4 0 0,51-9 0,-14-5 0,-1-3 0,66-35 0,75-57 0,-149 88 0,-10 7 0,-1-1 0,-1 0 0,0-2 0,-1-1 0,28-31 0,-38 35 0,0 1 0,-1-1 0,0-1 0,-2 0 0,1 0 0,-2-1 0,0 1 0,-1-1 0,6-31 0,-10 43 0,0 1 0,1-1 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,3-1 0,-2 1 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 0 0,-1 0 0,1 1 0,-1-2 0,3-6 0,-3 5 0,0 1 0,-1-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,-1 1 0,1-1 0,-1 0 0,0 0 0,-3-8 0,4 12 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 1 0,-3 1 0,-4 2 0,-1 0 0,1 0 0,0 1 0,1 0 0,-1 1 0,1 0 0,0 0 0,0 1 0,1 0 0,0 0 0,0 1 0,1 0 0,0 0 0,0 0 0,1 1 0,-5 9 0,-4 11 0,2 0 0,0 0 0,-14 59 0,26-87 0,-9 39 0,-6 43 0,14-73 0,0 0 0,1 0 0,0 0 0,0 0 0,1 0 0,0 0 0,1 0 0,0 0 0,0 0 0,6 11 0,-7-18 0,0 0 0,1-1 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0-1 0,-1 0 0,1 0 0,4-2 0,5-2 0,0-1 0,-1 0 0,1-1 0,-2 0 0,1-1 0,16-15 0,13-17 0,-3-2 0,-2-1 0,-1-2 0,32-57 0,-16 15 0,55-138 0,-88 182 0,-1 0 0,-3-1 0,-1-1 0,-3-1 0,-1 1 0,-2-1 0,-3 0 0,-1 0 0,-3-1 0,-1 1 0,-3 0 0,-1 0 0,-3 1 0,-14-47 0,-21-39 0,-75-157 0,-85-110 0,187 365 0,5 8 0,-2 0 0,0 1 0,-1 1 0,-2 0 0,-25-27 0,41 49 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-3 1 0,1 1 0,0 1 0,0-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,-1 5 0,-4 29 0,1 0 0,1 1 0,3 0 0,1 0 0,8 76 0,7 31-113,6 0 0,7-2-1,53 168 1,-40-190 48,5-2-1,6-2 1,129 220 0,-136-269 65,61 72 0,-87-120 0,1-1 0,1-1 0,0-1 0,2-1 0,0-1 0,48 28 0,-61-40 20,0-1-1,0 0 1,1-1-1,-1 1 1,1-2 0,-1 1-1,21 1 1,-26-4 7,1 0-1,-1 0 1,0-1-1,0 1 1,1-1-1,-1 0 1,0 0-1,0 0 1,0-1-1,0 0 1,0 1-1,0-1 1,-1-1 0,1 1-1,-1 0 1,1-1-1,-1 0 1,0 0-1,0 0 1,4-5-1,5-11-26,-1-1 0,-1 0 0,-1 0 0,-1-1 0,0 0 0,-2-1 0,6-34 0,7-17 0,21-49 0,-19 65 0,22-105 0,-42 160 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-3-2 0,1 3 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-6 1 0,-7 2 0,-1 1 0,1 0 0,0 2 0,-29 12 0,33-11 0,0 1 0,0 1 0,0 0 0,1 0 0,1 1 0,0 0 0,0 1 0,1 0 0,0 1 0,1 0 0,0 0 0,1 0 0,1 1 0,0 0 0,0 1 0,1-1 0,1 1 0,1 0 0,0 0 0,0 1 0,1-1 0,1 0 0,1 1 0,0-1 0,1 1 0,4 26 0,-4-38 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,5 2 0,-4-3 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,-1 0 0,1 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,4-3 0,4-2 0,-1-1 0,1 0 0,-1-1 0,-1 0 0,1-1 0,-2 1 0,14-18 0,2-10 0,-1-1 0,20-44 0,-4 7 0,-39 73 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1-1 0,1 1 0,0 1 0,0 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,3 4 0,23 27 0,-2 2 0,-1 1 0,26 49 0,10 15 0,-43-71 0,119 170 0,-108-161 0,2 0 0,68 62 0,-96-97 0,0 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,0 1 0,7-2 0,-7-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,1-1 0,-1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 0 0,1 0 0,0-4 0,11-33 0,-1 1 0,-2-1 0,6-60 0,1-136 0,-15 193 0,16-417 0,31-422 0,-40 809 0,-5 66 0,-1 20 0,13 259 0,-10-119 0,-4-112 0,56 692 0,-56-710 0,11 57 0,-12-74 0,1 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,1 1 0,0-1 0,0 0 0,4 5 0,-6-9 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,1-2 0,26-32 0,-15 11 0,-2-1 0,-1 0 0,-1-1 0,-1 0 0,-1 0 0,-1-1 0,-2 0 0,0 0 0,-2-1 0,0 1 0,-4-40 0,1 61 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,-1-1 0,1 0 0,-1 1 0,1 0 0,-1-1 0,0 1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 1 0,0-1 0,1 1 0,-1 0 0,0 0 0,-8-1 0,-10-2 0,0 1 0,-1 2 0,1 0 0,-42 2 0,39 1 0,3-2 0,-40 3 0,59-2 0,1 0 0,-1 1 0,1-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,1 0 0,-4 2 0,6-4 0,0 1 0,-1-1 0,1 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 1 0,19 8 0,24-2 0,-22-7 0,0-1 0,-1-1 0,1-1 0,-1 0 0,0-2 0,25-8 0,118-55 0,-131 53 0,-32 14 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 1 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,1 2 0,0 2 0,0 0 0,-1-1 0,0 1 0,0 1 0,0-1 0,-1 0 0,0 0 0,1 8 0,12 35 0,-10-42 0,0 1 0,0-1 0,1 0 0,-1-1 0,1 1 0,0-1 0,1 0 0,-1 0 0,1-1 0,0 0 0,0 0 0,12 6 0,-6-5 0,0 0 0,1-1 0,0-1 0,0 0 0,0 0 0,20 0 0,11-2 0,1-2 0,-1-2 0,51-11 0,-76 11 0,67-9 0,-1-4 0,0-3 0,85-33 0,-163 49 0,1 0 0,-1 0 0,1-1 0,-1-1 0,0 1 0,7-7 0,-13 10 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-2 0 0,-10-6 0,0 0 0,-1 1 0,0 0 0,0 1 0,-1 0 0,1 2 0,-24-4 0,-4-2 0,38 8 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 1 0,-4 2 0,4 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,0 1 0,0 0 0,1 0 0,-2 8 0,-2 6 0,1-1 0,1 1 0,1 0 0,0 0 0,2 0 0,0 0 0,1 0 0,1-1 0,8 38 0,-8-49 0,0 0 0,1 1 0,0-1 0,0 0 0,1 0 0,0-1 0,0 1 0,0-1 0,1 0 0,0 0 0,0 0 0,1-1 0,0 0 0,-1 0 0,2 0 0,-1-1 0,0 1 0,1-2 0,0 1 0,0-1 0,0 0 0,0 0 0,1-1 0,-1 0 0,1 0 0,-1-1 0,9 1 0,-6-1 0,0-1 0,1 1 0,-1-2 0,0 1 0,1-2 0,-1 1 0,0-1 0,0-1 0,0 0 0,-1 0 0,1-1 0,-1 0 0,1 0 0,-1-1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,9-10 0,-8 6 0,0-2 0,0 1 0,-1-1 0,0-1 0,-1 1 0,-1-1 0,0-1 0,-1 1 0,0-1 0,-1 0 0,-1 0 0,0 0 0,1-19 0,1-17 0,-3-1 0,-1 1 0,-11-81 0,9 157 0,0-22 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,2 6 0,-3-10 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0-1 0,11-20 0,-2-3 0,-2 0 0,0 0 0,-2 0 0,0-1 0,1-36 0,-5-134 0,-53-482 0,29 446 0,22 220 0,-100-744 0,98 740 0,1 2 0,0 0 0,-1 0 0,-1 0 0,0 0 0,-1 1 0,0 0 0,-1-1 0,0 2 0,-12-18 0,18 28 0,-1 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,-1 0 0,-1 4 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-3 11 0,-4 17 0,1 0 0,2 0 0,1 0 0,1 1 0,0 47 0,17 174 0,-1-150 0,5-1 0,5-1 0,4-1 0,5-1 0,4-2 0,4-1 0,4-2 0,5-1 0,4-3 0,3-3 0,5-1 0,3-4 0,4-2 0,4-3 0,2-3 0,98 78 0,-85-88 0,2-3 0,3-4 0,100 47 0,-181-101 0,-7-4 0,1 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,3 3 0,-7 5 0,-17 4 0,-43 12 0,-128 38 0,45-19 0,-92 42 0,5 10 0,4 10 0,-214 138 0,402-216 0,44-26 0,10-6 0,94-37 0,94-49 0,90-45-352,111-50-1058,129-51 409,339-132-1968,1193-456 2699,-2057 820 264,88-33 6,213-94 0,-303 128-5,0 0-1,-1-1 0,1 1 1,-1-1-1,1 0 0,-1 0 1,4-5-1,-8 8 11,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0-1,0-1 1,0 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0-1,-1 1 1,1-1 0,-71 2 1099,68-2-1047,-242 28 3197,185-21-10080</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink7.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-09-07T11:19:21.622"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">81 1266 24575,'-1'0'0,"1"0"0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,-2 4 0,-6 24 0,0 1 0,-5 45 0,-8 83-265,7 2 1,7 0-1,7 0 0,35 275 0,-25-373 265,2-1 0,3 0 0,2-1 0,39 88 0,-47-129 0,1 0 0,0-1 0,2-1 0,0 0 0,1 0 0,1-1 0,0-1 0,22 19 0,-23-24 0,1-1 0,1 0 0,-1 0 0,1-1 0,1-1 0,-1-1 0,1 0 0,0-1 0,1-1 0,27 4 0,-11-5-9,0-1 0,0-2 0,-1-1 0,1-2 0,0-1 0,-1-1 0,34-11 0,-10-2-160,0-1 0,-1-4 0,59-32 0,-45 16 131,-2-3 1,-2-3 0,-1-3-1,63-63 1,-60 44 46,-2-3 0,-4-2 1,59-90-1,-84 106 201,-2-1 1,35-85-1,-55 108-105,-1-1 0,-2 0 1,-1-1-1,-2 0 0,5-61 0,-12 87-105,0 0 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,0 1 0,-8-19 0,10 27-1,0 0 0,-1 0-1,1 0 1,0 0 0,-1 0 0,1 1-1,-1-1 1,1 0 0,-1 0 0,1 1-1,-1-1 1,0 0 0,1 1 0,-1-1-1,0 0 1,0 1 0,0-1 0,1 1-1,-1-1 1,0 1 0,0 0 0,0-1-1,0 1 1,0 0 0,0 0 0,1 0-1,-1-1 1,0 1 0,0 0 0,0 0-1,-1 1 1,-1 0 15,1 0 1,0 0-1,0 1 0,0-1 1,1 1-1,-1-1 0,0 1 0,0 0 1,1 0-1,-1-1 0,1 1 1,0 0-1,-2 3 0,-11 22 146,1 1 0,2 0 0,1 1 0,-10 43 0,-8 41-306,-26 224-1,48-257 74,3-1-1,4 1 1,19 138 0,-13-176 73,2-2 0,2 1 0,29 70 0,-31-92 0,0 0 0,1 0 0,2-1 0,-1 0 0,2-1 0,1 0 0,0-1 0,1-1 0,18 15 0,-27-24-3,1-1 1,1 0-1,-1-1 1,0 0 0,1 0-1,0-1 1,0 1-1,0-2 1,12 4-1,-16-6 8,-1 0-1,0 1 1,0-1-1,1 0 1,-1 0-1,0-1 1,0 1 0,1-1-1,-1 1 1,0-1-1,0 0 1,0 0-1,0-1 1,0 1-1,0-1 1,0 1-1,0-1 1,0 0-1,-1 0 1,1 0-1,-1 0 1,0-1-1,1 1 1,-1-1-1,0 1 1,2-5 0,4-7 53,-1-1 1,-1 1 0,-1-1 0,0 0 0,0 0 0,-2 0 0,0-1 0,1-15 0,1-129-101,-7 109 42,0 23 0,3-40 0,-1 68 0,-1-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,0-1 0,8 10 0,7 28 0,91 348 0,-75-258 0,-4-16 0,54 194 0,-67-264 0,-12-37 0,-1-8 0,-12-68 0,-101-640-515,62-10-1,49 704 516,-1 7 0,1-1 0,0 0 0,1 0 0,0 0 0,1 1 0,6-22 0,-7 31 7,-1 0 0,1 1 0,0-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,2 0 0,-1 1 21,0 0-1,-1 0 0,1 0 0,0 1 1,0-1-1,0 0 0,-1 1 0,1 0 1,0 0-1,0 0 0,-1 0 0,4 2 1,1 0 29,-1 1 0,1 1 1,-1-1-1,0 1 0,0 0 0,-1 0 1,1 1-1,7 11 0,-8-10-57,-1 1 0,0-1 0,-1 1 0,0 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,-1 1 0,0-1 0,0 14 0,-2-10 0,-1 0 0,1 1 0,-2-1 0,0 0 0,0-1 0,-1 1 0,-6 13 0,-6 5 0,-1-1 0,-2 0 0,-1-1 0,-40 44 0,27-39 0,26-27 0,0 0 0,0 1 0,0 1 0,1-1 0,-1 1 0,2 0 0,-8 14 0,12-21 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,1 0 0,38-7 0,-11-3 0,0-2 0,48-26 0,54-41 0,-108 64 0,-7 5 0,-1-1 0,0-1 0,-1 0 0,-1-1 0,21-23 0,-28 26 0,0 0 0,0 0 0,-1 0 0,0-1 0,-1 0 0,0-1 0,-1 1 0,0-1 0,4-22 0,-7 32 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,2-1 0,-1 1 0,0-1 0,-1 1 0,0 0 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 0 0,-1 0 0,3-5 0,-3 4 0,0 0 0,0-1 0,0 1 0,0 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,-1 1 0,0 0 0,-1-6 0,1 8 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,-2 2 0,-2 0 0,-1 1 0,0 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,0 1 0,1 0 0,-1 0 0,1 0 0,0 1 0,1-1 0,-1 1 0,1 1 0,0-1 0,-3 7 0,-3 8 0,1 0 0,1 0 0,-11 43 0,19-63 0,-7 28 0,-3 32 0,9-54 0,0 0 0,1 0 0,-1 1 0,2-1 0,-1 0 0,1 0 0,1 1 0,-1-1 0,1 0 0,3 9 0,-4-14 0,0-1 0,0 1 0,0 0 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,3-1 0,4-2 0,-1 0 0,1-1 0,-1 0 0,0 0 0,-1-1 0,13-11 0,9-12 0,-2-1 0,-1-1 0,-2-2 0,24-41 0,-12 10 0,41-99 0,-64 132 0,-2-1 0,-1 0 0,-2-1 0,-1 0 0,-2 0 0,0 0 0,-3-1 0,-1 1 0,-1-1 0,-2 0 0,-1 1 0,-2 0 0,-1-1 0,-11-32 0,-15-30 0,-54-113 0,-63-81 0,137 266 0,3 6 0,-1 0 0,0 1 0,-2 0 0,0 0 0,-18-19 0,29 35 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-2 1 0,1 0 0,0 0 0,0 1 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1 3 0,-4 21 0,2 1 0,0 0 0,2 0 0,2 0 0,5 55 0,5 23-113,5 0 0,4-1-1,40 122 1,-30-139 48,4-1-1,3-2 1,95 161 0,-99-196 65,45 53 0,-64-89 0,1 0 0,0 0 0,1-1 0,1-1 0,0-1 0,35 21 0,-45-30 20,1 1-1,0-2 1,-1 1-1,1-1 1,0 0 0,0 0-1,15 1 1,-19-3 7,0 0-1,0 0 1,0 0-1,0-1 1,1 1-1,-1-1 1,0 0-1,0 0 1,-1 0-1,1 0 1,0 0-1,0-1 1,0 1 0,-1-1-1,1 0 1,-1 0-1,1 0 1,-1 0-1,0 0 1,3-4-1,4-8-26,-1 0 0,-1-1 0,0 0 0,-1 0 0,-1 0 0,0-1 0,4-25 0,4-12 0,16-36 0,-14 48 0,17-77 0,-32 116 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,-2-1 0,0 1 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-4 1 0,-6 1 0,0 1 0,0 0 0,0 1 0,-20 10 0,22-9 0,2 1 0,-1 0 0,1 0 0,0 1 0,0 0 0,1 1 0,0 0 0,0 0 0,1 0 0,0 1 0,0 0 0,1 0 0,0 0 0,1 1 0,0 0 0,1 0 0,-1 0 0,2 0 0,0 0 0,0 0 0,1 1 0,0-1 0,0 1 0,2-1 0,-1 1 0,4 19 0,-3-28 0,-1 0 0,0 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1-1 0,1 0 0,0 1 0,-1-1 0,5 2 0,-5-2 0,1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 0 0,0 1 0,3-3 0,3-2 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0-1 0,-1 1 0,10-13 0,1-7 0,0-1 0,14-31 0,-3 3 0,-27 55 0,-1-1 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 1 0,1 2 0,17 20 0,0 1 0,-2 1 0,19 36 0,7 11 0,-30-52 0,85 124 0,-78-117 0,2-1 0,49 46 0,-70-71 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1-1 0,0 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 0 0,0 1 0,0-1 0,5-1 0,-5 0 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,1-3 0,8-23 0,-2-1 0,-1 0 0,5-43 0,1-100 0,-12 141 0,12-303 0,22-307 0,-27 588 0,-6 48 0,0 15 0,10 188 0,-8-86 0,-2-82 0,40 503 0,-40-516 0,7 41 0,-8-53 0,0 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,4 3 0,-6-5 0,1-1 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 1 0,0-1 0,-1 1 0,2-2 0,18-22 0,-11 7 0,0 0 0,-2-1 0,0 0 0,-2 0 0,0-1 0,0 0 0,-2 1 0,0-1 0,-2-1 0,0 1 0,-2-29 0,0 44 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,-1 1 0,-5-1 0,-8-2 0,0 1 0,0 1 0,0 1 0,-30 1 0,28 1 0,2-1 0,-29 0 0,43 1 0,1-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 0 0,-2 3 0,4-4 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,15 7 0,17-2 0,-16-5 0,0 0 0,0-2 0,-1 0 0,1 0 0,-1-2 0,18-5 0,86-41 0,-95 39 0,-22 11 0,-1-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,1 2 0,0 0 0,0 0 0,0 1 0,0 0 0,-1-1 0,0 1 0,0 0 0,0 0 0,1 5 0,8 26 0,-8-30 0,1-1 0,0 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,1-1 0,-1 0 0,1 0 0,7 4 0,-3-3 0,0-1 0,0 0 0,1 0 0,-1-1 0,1 0 0,13 0 0,10-1 0,-1-2 0,1-2 0,36-6 0,-56 7 0,50-7 0,-1-3 0,-1-2 0,63-23 0,-119 35 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0-1 0,5-4 0,-9 8 0,0-1 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 1 0,1 0 0,-2-1 0,-8-5 0,0 1 0,0 1 0,0 0 0,0 0 0,-1 1 0,1 0 0,-18-2 0,-2-1 0,27 5 0,0 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,-2 2 0,2 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,1 1 0,0-1 0,-2 7 0,0 3 0,0 1 0,1-1 0,0 1 0,1 0 0,1 0 0,0-1 0,1 1 0,0 0 0,7 26 0,-7-34 0,1-1 0,0 0 0,0 0 0,0 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 0 0,-1 0 0,7 1 0,-5-2 0,1 1 0,-1-1 0,1 0 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 0 0,-1-1 0,0 1 0,-1-1 0,1-1 0,0 1 0,-1-1 0,0 0 0,0-1 0,0 1 0,6-8 0,-5 4 0,0 0 0,-1 0 0,0-1 0,-1 0 0,1 0 0,-2-1 0,0 1 0,0-1 0,0 0 0,-1 0 0,-1-1 0,0 1 0,1-14 0,1-12 0,-3-1 0,0 0 0,-8-58 0,6 114 0,0-16 0,0 0 0,1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,2 6 0,-2-8 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,9-14 0,-3-2 0,-1-1 0,0 1 0,-1-1 0,-1 0 0,2-26 0,-4-99 0,-40-349 0,23 325 0,15 159 0,-72-542 0,71 540 0,0 0 0,1 0 0,-2 1 0,1 0 0,-1-1 0,-1 1 0,1 0 0,-2 0 0,1 1 0,-9-13 0,12 21 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,-2 2 0,0 1 0,1-1 0,0 1 0,0 0 0,0 0 0,-3 7 0,-2 13 0,0 0 0,2 0 0,0 0 0,2 1 0,0 34 0,11 126 0,0-109 0,4 0 0,3-1 0,3-1 0,4-1 0,3 0 0,2-2 0,4-1 0,3-1 0,3-2 0,3-2 0,3-2 0,2-1 0,3-3 0,2-1 0,3-3 0,71 57 0,-63-64 0,3-2 0,1-3 0,73 34 0,-131-74 0,-6-2 0,1 0 0,0 0 0,0-1 0,0 2 0,0-1 0,-1 0 0,1 0 0,0 0 0,1 3 0,-4 3 0,-13 3 0,-31 9 0,-93 27 0,32-13 0,-66 31 0,3 6 0,3 8 0,-155 100 0,292-157 0,32-18 0,7-5 0,68-27 0,70-37 0,64-31-352,81-37-1058,94-37 409,246-95-1968,869-333 2699,-1497 597 264,64-25 6,155-67 0,-220 92-5,-1 1-1,0-1 0,1 0 1,-1 0-1,0 0 0,0 0 1,3-4-1,-6 6 11,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1-1 0,1 1-1,0 0 1,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0-1,-1 0 1,1 1 0,-52 0 1099,50-1-1047,-176 21 3197,134-16-10080</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2077,26 +2346,26 @@
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="20"/>
-      <c r="C4" s="108" t="s">
+      <c r="C4" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="109"/>
-      <c r="E4" s="112" t="s">
+      <c r="D4" s="110"/>
+      <c r="E4" s="113" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="109" t="s">
+      <c r="F4" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="109"/>
+      <c r="G4" s="110"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="21"/>
-      <c r="C5" s="110"/>
-      <c r="D5" s="111"/>
-      <c r="E5" s="113"/>
-      <c r="F5" s="111"/>
-      <c r="G5" s="111"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="112"/>
+      <c r="E5" s="114"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="112"/>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -2514,6 +2783,54 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C399C8E1-E30A-4896-9972-62C0E4F77BE1}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="B5:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="48" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2718,10 +3035,10 @@
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="114" t="s">
+      <c r="B11" s="115" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="114"/>
+      <c r="C11" s="115"/>
       <c r="D11" s="31" t="s">
         <v>40</v>
       </c>
@@ -2741,10 +3058,10 @@
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="114" t="s">
+      <c r="B12" s="115" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="114"/>
+      <c r="C12" s="115"/>
       <c r="D12" s="31" t="s">
         <v>40</v>
       </c>
@@ -3077,17 +3394,17 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C3" s="115" t="s">
+      <c r="C3" s="116" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="115"/>
-      <c r="E3" s="115"/>
-      <c r="L3" s="115" t="s">
+      <c r="D3" s="116"/>
+      <c r="E3" s="116"/>
+      <c r="L3" s="116" t="s">
         <v>92</v>
       </c>
-      <c r="M3" s="115"/>
-      <c r="N3" s="115"/>
-      <c r="O3" s="115"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
       <c r="Q3" s="76" t="s">
         <v>94</v>
       </c>
@@ -3865,7 +4182,7 @@
     <mergeCell ref="L3:O3"/>
   </mergeCells>
   <conditionalFormatting sqref="K15:O17 A15:J16 B17:J17 B4:O14 B18:O38">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -3904,11 +4221,11 @@
       <c r="E3" s="81">
         <v>46121</v>
       </c>
-      <c r="H3" s="116" t="s">
+      <c r="H3" s="117" t="s">
         <v>109</v>
       </c>
-      <c r="I3" s="117"/>
-      <c r="J3" s="118"/>
+      <c r="I3" s="118"/>
+      <c r="J3" s="119"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="84"/>
@@ -4059,53 +4376,173 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E2123E-1D13-46F0-9B4A-A5272E85634C}">
-  <dimension ref="D2:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F945C220-D127-489B-A05F-24B39A2383B1}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="B1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="120" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" t="s">
+        <v>132</v>
+      </c>
       <c r="D5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="4:4" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" t="s">
+        <v>126</v>
+      </c>
       <c r="D8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>98</v>
-      </c>
-    </row>
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="121"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" t="s">
+        <v>135</v>
+      </c>
+      <c r="D13" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" t="s">
+        <v>133</v>
+      </c>
+      <c r="D14" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="78" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D16" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C4:C27">
+    <sortCondition ref="C1:C27"/>
+  </sortState>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6C46C7F-8851-4D1E-AAA5-68FB05373326}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
   <dimension ref="A2:L22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4203,22 +4640,6 @@
       <c r="B11" s="105"/>
       <c r="C11" s="106"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="E13" s="119" t="s">
-        <v>123</v>
-      </c>
-      <c r="F13" s="119"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="F15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="F16" t="s">
-        <v>124</v>
-      </c>
-    </row>
     <row r="17" spans="4:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D18" s="82"/>
@@ -4258,68 +4679,92 @@
       <c r="F22" s="87"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="F3:L3"/>
-    <mergeCell ref="E13:F13"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E2123E-1D13-46F0-9B4A-A5272E85634C}">
+  <dimension ref="D2:D9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F945C220-D127-489B-A05F-24B39A2383B1}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C399C8E1-E30A-4896-9972-62C0E4F77BE1}">
-  <sheetPr>
-    <tabColor rgb="FFFF0000"/>
-  </sheetPr>
-  <dimension ref="B5:C15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0E9D792-2517-4CE8-8D18-28421B01A876}">
+  <dimension ref="A8:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="48" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>101</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>103</v>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="108" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="108"/>
+      <c r="C8" s="108"/>
+      <c r="D8" s="108"/>
+      <c r="E8" s="108"/>
+      <c r="F8" s="108"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
+  <mergeCells count="1">
+    <mergeCell ref="A8:F8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Payment And Student reg id getting is ok Chhecked also coreclty in the local wanna host these coreclty
</commit_message>
<xml_diff>
--- a/Sql/HD prob.xlsx
+++ b/Sql/HD prob.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ims-october-bkps\Sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8624F0B-8815-4616-B06B-3211184AD3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D364F6C9-73EB-4B71-9F24-B212262EBE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="630" windowWidth="20730" windowHeight="11040" tabRatio="692" firstSheet="5" activeTab="5" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="692" firstSheet="7" activeTab="8" xr2:uid="{D32FFA46-9C2E-4324-9790-4976D8E4A0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -18,11 +18,12 @@
     <sheet name="Payment Duplicate error fix" sheetId="4" state="hidden" r:id="rId3"/>
     <sheet name="Transfered  Progression Checkin" sheetId="5" state="hidden" r:id="rId4"/>
     <sheet name="POS  and PAGE UPDATE" sheetId="7" state="hidden" r:id="rId5"/>
-    <sheet name="Induction re-arrange" sheetId="13" r:id="rId6"/>
-    <sheet name="re register" sheetId="12" r:id="rId7"/>
+    <sheet name="Induction re-arrange" sheetId="13" state="hidden" r:id="rId6"/>
+    <sheet name="re register" sheetId="12" state="hidden" r:id="rId7"/>
     <sheet name="HD RESULT" sheetId="2" r:id="rId8"/>
     <sheet name="New ID Order Missing " sheetId="14" r:id="rId9"/>
-    <sheet name="Sheet2" sheetId="6" state="hidden" r:id="rId10"/>
+    <sheet name="Sheet3" sheetId="15" r:id="rId10"/>
+    <sheet name="Sheet2" sheetId="6" state="hidden" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="146">
   <si>
     <t>Re-sit</t>
   </si>
@@ -532,6 +533,21 @@
   </si>
   <si>
     <t>07-09-2026 data</t>
+  </si>
+  <si>
+    <t>ajax/</t>
+  </si>
+  <si>
+    <t>payment_withheld.php</t>
+  </si>
+  <si>
+    <t>WithHeld Data coreclty</t>
+  </si>
+  <si>
+    <t>induction_DB_folder\fetch_induction_email_templates.php</t>
+  </si>
+  <si>
+    <t>email body template active inactive shows</t>
   </si>
 </sst>
 </file>
@@ -1076,7 +1092,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1236,10 +1252,11 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1275,8 +1292,12 @@
     <xf numFmtId="0" fontId="10" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1700,8 +1721,8 @@
       <xdr:row>14</xdr:row>
       <xdr:rowOff>164145</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="4" name="Ink 3">
@@ -1720,7 +1741,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="4" name="Ink 3">
@@ -1770,8 +1791,8 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>47685</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="2" name="Ink 1">
@@ -1790,7 +1811,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="2" name="Ink 1">
@@ -2346,26 +2367,26 @@
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="20"/>
-      <c r="C4" s="109" t="s">
+      <c r="C4" s="110" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="110"/>
-      <c r="E4" s="113" t="s">
+      <c r="D4" s="111"/>
+      <c r="E4" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="110" t="s">
+      <c r="F4" s="111" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="110"/>
+      <c r="G4" s="111"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="21"/>
-      <c r="C5" s="111"/>
-      <c r="D5" s="112"/>
-      <c r="E5" s="114"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="112"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -2787,6 +2808,15 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99CCEDAB-CE43-4A7E-B09A-9247E540F366}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C399C8E1-E30A-4896-9972-62C0E4F77BE1}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
@@ -3035,10 +3065,10 @@
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="115" t="s">
+      <c r="B11" s="116" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="115"/>
+      <c r="C11" s="116"/>
       <c r="D11" s="31" t="s">
         <v>40</v>
       </c>
@@ -3058,10 +3088,10 @@
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="115" t="s">
+      <c r="B12" s="116" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="115"/>
+      <c r="C12" s="116"/>
       <c r="D12" s="31" t="s">
         <v>40</v>
       </c>
@@ -3394,17 +3424,17 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C3" s="116" t="s">
+      <c r="C3" s="117" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="L3" s="116" t="s">
+      <c r="D3" s="117"/>
+      <c r="E3" s="117"/>
+      <c r="L3" s="117" t="s">
         <v>92</v>
       </c>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
-      <c r="O3" s="116"/>
+      <c r="M3" s="117"/>
+      <c r="N3" s="117"/>
+      <c r="O3" s="117"/>
       <c r="Q3" s="76" t="s">
         <v>94</v>
       </c>
@@ -4221,11 +4251,11 @@
       <c r="E3" s="81">
         <v>46121</v>
       </c>
-      <c r="H3" s="117" t="s">
+      <c r="H3" s="118" t="s">
         <v>109</v>
       </c>
-      <c r="I3" s="118"/>
-      <c r="J3" s="119"/>
+      <c r="I3" s="119"/>
+      <c r="J3" s="120"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="84"/>
@@ -4388,7 +4418,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="120" t="s">
+      <c r="B1" s="107" t="s">
         <v>140</v>
       </c>
     </row>
@@ -4443,9 +4473,6 @@
       <c r="D8" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="121"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="78" t="s">
@@ -4560,15 +4587,15 @@
       <c r="C3" s="83" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="107" t="s">
+      <c r="F3" s="121" t="s">
         <v>120</v>
       </c>
-      <c r="G3" s="107"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="107"/>
-      <c r="K3" s="107"/>
-      <c r="L3" s="107"/>
+      <c r="G3" s="121"/>
+      <c r="H3" s="121"/>
+      <c r="I3" s="121"/>
+      <c r="J3" s="121"/>
+      <c r="K3" s="121"/>
+      <c r="L3" s="121"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="101"/>
@@ -4735,13 +4762,46 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0E9D792-2517-4CE8-8D18-28421B01A876}">
-  <dimension ref="A8:F11"/>
+  <dimension ref="A3:N15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="48.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H4" s="82"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="83"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H5" s="84"/>
+      <c r="I5" s="108" t="s">
+        <v>143</v>
+      </c>
+      <c r="J5" s="108"/>
+      <c r="K5" s="108"/>
+      <c r="L5" s="108"/>
+      <c r="M5" s="108"/>
+      <c r="N5" s="109"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H6" s="84"/>
+      <c r="N6" s="85"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H7" s="84"/>
+      <c r="I7" t="s">
+        <v>141</v>
+      </c>
+      <c r="N7" s="85"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="108" t="s">
         <v>123</v>
       </c>
@@ -4750,20 +4810,49 @@
       <c r="D8" s="108"/>
       <c r="E8" s="108"/>
       <c r="F8" s="108"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H8" s="84"/>
+      <c r="I8" t="s">
+        <v>142</v>
+      </c>
+      <c r="N8" s="85"/>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H9" s="86"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
+      <c r="L9" s="44"/>
+      <c r="M9" s="44"/>
+      <c r="N9" s="87"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>124</v>
       </c>
     </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I13" s="122" t="s">
+        <v>145</v>
+      </c>
+      <c r="J13" s="122"/>
+      <c r="K13" s="122"/>
+      <c r="L13" s="122"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>144</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A8:F8"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="I13:L13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>